<commit_message>
Refresh CTT_NL_Sources from main and make database duplicate-check mandatory
Pulled the user's refreshed CTT_NL_Sources.xlsx from origin/main and
regenerated CTT_NL_Sources.csv from it. The refresh had dropped the
source-name column entirely and mangled one hyperlink into an
Office-Online redirect; recovered both by matching URLs against the
previous CSV rather than trusting the new sheet blind. One genuine
addition: Ryan's press room.

Also makes the CTT_NL_Database.csv duplicate-check mandatory for every
candidate (not just suspicious-looking ones) per explicit instruction,
and corrects the skill's "no shell/script execution" assumption, which
isn't true in this session (Bash + Python/openpyxl are available and
needed for reliable xlsx hyperlink extraction).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011o6uZop4h8MZcvQcamNxqZ
</commit_message>
<xml_diff>
--- a/CTT_NL_Sources.xlsx
+++ b/CTT_NL_Sources.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://trten-my.sharepoint.com/personal/prathika_gowdamn_thomsonreuters_com/Documents/Claude/Corporates_Newsletter/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\6135878\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="24" documentId="11_F25DC773A252ABDACC10486D995B54765BDE5902" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1780D5D9-C0F3-4218-A61D-C56CA0089B1E}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{003DACC5-99CB-45FF-9A2A-B350EC1AE882}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="3">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="4">
   <si>
     <t>Press</t>
   </si>
@@ -45,6 +45,9 @@
   </si>
   <si>
     <t>Link</t>
+  </si>
+  <si>
+    <t>Ryan</t>
   </si>
 </sst>
 </file>
@@ -373,7 +376,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:A105"/>
+  <dimension ref="A1:A106"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.35">
@@ -899,6 +902,11 @@
     <row r="105" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A105" s="1" t="s">
         <v>2</v>
+      </c>
+    </row>
+    <row r="106" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A106" s="1" t="s">
+        <v>3</v>
       </c>
     </row>
   </sheetData>
@@ -1008,6 +1016,7 @@
     <hyperlink ref="A103" r:id="rId103" display="https://www.linkedin.com/company/resilinc/posts/?feedView=all&amp;viewAsMember=true" xr:uid="{A3CE0775-E79F-4559-9AFE-97C955AB2196}"/>
     <hyperlink ref="A104" r:id="rId104" display="https://www.linkedin.com/company/taxera/posts/?feedView=all&amp;viewAsMember=true" xr:uid="{70D861A6-F8C6-4C35-BC1D-24B4A5711778}"/>
     <hyperlink ref="A105" r:id="rId105" display="https://www.linkedin.com/company/pairsoft/posts/?feedView=all" xr:uid="{61288785-74A3-4AF4-850A-065B38B7BEE2}"/>
+    <hyperlink ref="A106" r:id="rId106" xr:uid="{F728FD77-964F-4255-B638-6E575CC52CA0}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>